<commit_message>
ajuste leitura parquet e alteracao descrição de jornadas
</commit_message>
<xml_diff>
--- a/data/jornadas_comerciais_poc.xlsx
+++ b/data/jornadas_comerciais_poc.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="307">
   <si>
     <t>Jornada_ID</t>
   </si>
@@ -231,33 +231,18 @@
     <t>Carteira01</t>
   </si>
   <si>
-    <t>Revisão completa da carteira avaliando diversificação, risco, liquidez e aderência ao perfil do cliente. Pode gerar sugestões envolvendo fundos multimercado, ETFs, renda fixa, fundos internacionais ou alternativos.</t>
-  </si>
-  <si>
     <t>Carteira02</t>
   </si>
   <si>
-    <t>Ajuste dos pesos entre classes de ativos após movimentos de mercado para retornar à alocação estratégica. Pode envolver venda parcial de ações, compra de renda fixa, ETFs ou multimercados.</t>
-  </si>
-  <si>
     <t>Carteira03</t>
   </si>
   <si>
-    <t>Cliente possui concentração excessiva em um ativo, empresa ou setor. A estratégia envolve diversificação progressiva utilizando fundos, ETFs globais, FIIs ou crédito privado.</t>
-  </si>
-  <si>
     <t>Carteira04</t>
   </si>
   <si>
-    <t>Apresentar importância da diversificação geográfica e proteção cambial. Produtos incluem ETFs globais, BDRs, fundos internacionais ou multimercados globais.</t>
-  </si>
-  <si>
     <t>Carteira05</t>
   </si>
   <si>
-    <t>Reorganização de investimentos visando reduzir impacto tributário. Pode envolver previdência, ETFs, fundos exclusivos ou estratégias de compensação de prejuízos.</t>
-  </si>
-  <si>
     <t>Carteira06</t>
   </si>
   <si>
@@ -267,9 +252,6 @@
     <t>Organização</t>
   </si>
   <si>
-    <t>Reduzir excesso de produtos ou estruturas complexas, consolidando em fundos multimercado, ETFs amplos ou estratégias core.</t>
-  </si>
-  <si>
     <t>Carteira07</t>
   </si>
   <si>
@@ -279,9 +261,6 @@
     <t>Acompanhamento</t>
   </si>
   <si>
-    <t>Revisão periódica para validar aderência da carteira aos objetivos do cliente considerando mudanças de cenário.</t>
-  </si>
-  <si>
     <t>Carteira08</t>
   </si>
   <si>
@@ -291,18 +270,12 @@
     <t>Geração de Renda</t>
   </si>
   <si>
-    <t>Ajustar carteira buscando maior geração de fluxo recorrente com FIIs, debêntures, crédito privado ou fundos de dividendos.</t>
-  </si>
-  <si>
     <t>Carteira09</t>
   </si>
   <si>
     <t>Proteção de Patrimônio</t>
   </si>
   <si>
-    <t>Introdução de ativos defensivos como renda fixa indexada à inflação, ouro, multimercados macro ou estratégias long/short.</t>
-  </si>
-  <si>
     <t>Carteira10</t>
   </si>
   <si>
@@ -312,9 +285,6 @@
     <t>Estruturação</t>
   </si>
   <si>
-    <t>Reorganizar carteira em núcleo estável com ETFs ou fundos amplos e satélites táticos para oportunidades específicas.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro01</t>
   </si>
   <si>
@@ -324,21 +294,12 @@
     <t>Investimento</t>
   </si>
   <si>
-    <t>Cliente recebeu liquidez relevante e busca direcionamento. Estruturação pode envolver renda fixa, multimercados, ações ou ETFs.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro02</t>
   </si>
   <si>
-    <t>Recursos provenientes de resgate precisam ser redirecionados para novas oportunidades alinhadas ao cenário.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro03</t>
   </si>
   <si>
-    <t>Excesso de caixa parado. Sugestões incluem fundos DI, CDB liquidez diária ou fundos de crédito.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro04</t>
   </si>
   <si>
@@ -348,9 +309,6 @@
     <t>Planejamento de Investimento</t>
   </si>
   <si>
-    <t>Cliente recebeu bônus corporativo e deseja investir estrategicamente.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro05</t>
   </si>
   <si>
@@ -360,9 +318,6 @@
     <t>Alocação Patrimonial</t>
   </si>
   <si>
-    <t>Cliente recebeu grande liquidez após venda de negócio ou imóvel e precisa estruturar carteira.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro06</t>
   </si>
   <si>
@@ -372,9 +327,6 @@
     <t>Gestão de Liquidez</t>
   </si>
   <si>
-    <t>Organizar retiradas programadas mantendo rentabilidade adequada.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro07</t>
   </si>
   <si>
@@ -384,9 +336,6 @@
     <t>Ajuste Financeiro</t>
   </si>
   <si>
-    <t>Mudança no fluxo de renda exige revisão da carteira.</t>
-  </si>
-  <si>
     <t>FluxoFinanceiro08</t>
   </si>
   <si>
@@ -396,15 +345,9 @@
     <t>Proteção Financeira</t>
   </si>
   <si>
-    <t>Estruturar reserva em produtos de alta liquidez como Tesouro Selic, CDB diário ou fundos DI.</t>
-  </si>
-  <si>
     <t>Produto01</t>
   </si>
   <si>
-    <t>Apresentação de produto alinhado ao perfil do cliente e ao cenário de mercado, explicando estratégia, riscos, horizonte e papel dentro da carteira.</t>
-  </si>
-  <si>
     <t>Produto02</t>
   </si>
   <si>
@@ -501,9 +444,6 @@
     <t>Atualização</t>
   </si>
   <si>
-    <t>Explicar mudanças no cenário econômico e impactos na carteira sugerindo possíveis ajustes estratégicos.</t>
-  </si>
-  <si>
     <t>Cenario02</t>
   </si>
   <si>
@@ -558,9 +498,6 @@
     <t>Relacionamento01</t>
   </si>
   <si>
-    <t>Interação focada em fortalecer vínculo, manter proximidade e gerar oportunidades de conversa sobre investimentos.</t>
-  </si>
-  <si>
     <t>Relacionamento02</t>
   </si>
   <si>
@@ -591,9 +528,6 @@
     <t>Planejamento01</t>
   </si>
   <si>
-    <t>Estruturação de investimentos considerando horizonte, objetivos e perfil do cliente.</t>
-  </si>
-  <si>
     <t>Planejamento02</t>
   </si>
   <si>
@@ -657,9 +591,6 @@
     <t>Risco01</t>
   </si>
   <si>
-    <t>Ajuste da carteira para proteger patrimônio e reduzir exposição a riscos específicos.</t>
-  </si>
-  <si>
     <t>Risco02</t>
   </si>
   <si>
@@ -696,9 +627,6 @@
     <t>Correção</t>
   </si>
   <si>
-    <t>Discussão sobre desempenho da carteira e possíveis ajustes estratégicos.</t>
-  </si>
-  <si>
     <t>Performance02</t>
   </si>
   <si>
@@ -732,9 +660,6 @@
     <t>Educação Financeira</t>
   </si>
   <si>
-    <t>Conteúdo educacional para ajudar o cliente a entender melhor conceitos de investimento.</t>
-  </si>
-  <si>
     <t>Educacional02</t>
   </si>
   <si>
@@ -771,9 +696,6 @@
     <t>Regulatório</t>
   </si>
   <si>
-    <t>Interação necessária para manter dados atualizados e garantir aderência regulatória.</t>
-  </si>
-  <si>
     <t>Compliance02</t>
   </si>
   <si>
@@ -784,6 +706,240 @@
   </si>
   <si>
     <t>Validação de Perfil de Risco</t>
+  </si>
+  <si>
+    <t>Diagnóstico amplo da carteira para identificar concentração, liquidez, aderência ao perfil e oportunidades de melhoria na alocação estratégica do cliente.</t>
+  </si>
+  <si>
+    <t>Revisão da alocação atual para corrigir desvios de peso entre classes de ativos e recompor a carteira conforme a estratégia originalmente definida.</t>
+  </si>
+  <si>
+    <t>Abordagem focada em reduzir exposição excessiva a um ativo, emissor ou setor, diminuindo risco específico sem perder o racional de investimento.</t>
+  </si>
+  <si>
+    <t>Conversa voltada a ampliar a parcela internacional da carteira, trazendo diversificação geográfica, cambial e acesso a mercados globais.</t>
+  </si>
+  <si>
+    <t>Revisão da estrutura da carteira com foco em eficiência tributária, avaliando produtos, prazos e alternativas que possam melhorar o retorno líquido.</t>
+  </si>
+  <si>
+    <t>Proposta para enxugar uma carteira excessivamente fragmentada, consolidando posições e deixando a alocação mais clara, acompanhável e eficiente.</t>
+  </si>
+  <si>
+    <t>Contato periódico para revisar se a carteira continua adequada aos objetivos, ao perfil do cliente e ao cenário de mercado mais recente.</t>
+  </si>
+  <si>
+    <t>Ajuste de carteira com foco em aumentar geração de renda recorrente, priorizando instrumentos que reforcem fluxo mensal ou previsibilidade de caixa.</t>
+  </si>
+  <si>
+    <t>Estratégia defensiva para proteger patrimônio em cenários de maior incerteza, com ênfase em preservação de capital e redução de vulnerabilidades.</t>
+  </si>
+  <si>
+    <t>Estruturação da carteira em um núcleo principal mais estável e posições satélite mais táticas, equilibrando consistência e captura de oportunidades.</t>
+  </si>
+  <si>
+    <t>Direcionamento para investir novos recursos recém-disponibilizados, definindo alocação inicial conforme prazo, perfil e objetivos do cliente.</t>
+  </si>
+  <si>
+    <t>Recomendação para realocar valores provenientes de resgates, evitando caixa ocioso e reposicionando os recursos em alternativas mais adequadas.</t>
+  </si>
+  <si>
+    <t>Abordagem para reduzir excesso de caixa parado em conta, buscando melhor rentabilidade sem comprometer a liquidez necessária do cliente.</t>
+  </si>
+  <si>
+    <t>Planejamento de investimento para valores recebidos em bônus, transformando um evento pontual de renda em construção patrimonial mais eficiente.</t>
+  </si>
+  <si>
+    <t>Estruturação de alocação após venda de empresa, imóvel ou outro ativo relevante, com atenção especial a liquidez, risco e diversificação.</t>
+  </si>
+  <si>
+    <t>Organização da carteira para suportar saques planejados, equilibrando liquidez, previsibilidade e manutenção do patrimônio ao longo do tempo.</t>
+  </si>
+  <si>
+    <t>Revisão financeira para adaptar aportes, liquidez e risco da carteira a uma nova realidade de renda mensal do cliente.</t>
+  </si>
+  <si>
+    <t>Montagem ou reforço da reserva de emergência com produtos adequados para liquidez rápida, baixa volatilidade e proteção financeira imediata.</t>
+  </si>
+  <si>
+    <t>Jornada comercial com objetivo de oferecer um COE, explicando a estrutura, os cenários de retorno, o prazo, os riscos e o papel do produto na carteira.</t>
+  </si>
+  <si>
+    <t>Jornada comercial com objetivo de oferecer um CDB, destacando taxa, prazo, liquidez, risco de crédito e aderência à parcela de renda fixa do cliente.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer um fundo multimercado como solução de diversificação, gestão ativa e busca de retorno em diferentes cenários de mercado.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer um fundo imobiliário, explorando potencial de renda, exposição ao setor imobiliário e papel do produto na geração de fluxo.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer um ETF internacional, reforçando diversificação global, acesso a bolsas externas e eficiência operacional na alocação.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer uma estratégia de private equity, ressaltando horizonte mais longo, iliquidez e potencial de valorização em ativos alternativos.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer exposição a criptoativos, contextualizando volatilidade, tese de diversificação e tamanho adequado da posição dentro da carteira.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer debêntures, explicando risco de crédito, prazo, indexador e potencial de retorno adicional dentro da renda fixa.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer previdência privada, conectando benefício sucessório, eficiência tributária e planejamento de longo prazo do cliente.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer fundo de ações, apresentando estratégia de gestão, perfil de volatilidade e adequação ao objetivo de crescimento patrimonial.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer fundo cambial, mostrando como a estratégia pode proteger parte do patrimônio em cenários de oscilação do dólar.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer LCI ou LCA, enfatizando isenção fiscal, prazo, liquidez e papel tático na composição da renda fixa.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer um fundo quantitativo, explicando o processo sistemático de investimento e o diferencial da estratégia baseada em modelos.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer fundo de dividendos, alinhando a estratégia à busca por renda recorrente, qualidade de empresas e disciplina de distribuição.</t>
+  </si>
+  <si>
+    <t>Jornada para oferecer exposição a ouro ou commodities, destacando proteção, diversificação e comportamento diferenciado em cenários de estresse.</t>
+  </si>
+  <si>
+    <t>Explicar o cenário macroeconômico atual e traduzir seus efeitos práticos sobre juros, bolsa, inflação, câmbio e posicionamento da carteira.</t>
+  </si>
+  <si>
+    <t>Explicar como uma mudança de política monetária altera expectativa de juros, preço dos ativos e decisões de alocação em renda fixa e risco.</t>
+  </si>
+  <si>
+    <t>Contato preventivo em momentos de maior oscilação para contextualizar a volatilidade, reduzir reação emocional e reforçar disciplina de longo prazo.</t>
+  </si>
+  <si>
+    <t>Atualização sobre mudanças no cenário internacional e seus reflexos sobre bolsa, dólar, commodities e oportunidades fora do mercado doméstico.</t>
+  </si>
+  <si>
+    <t>Conversa focada em alta da inflação, mostrando impactos sobre poder de compra, renda fixa real e necessidade de proteção da carteira.</t>
+  </si>
+  <si>
+    <t>Abordagem após queda da bolsa para reavaliar posição do cliente, separar ruído de fundamento e discutir ajustes ou manutenção de estratégia.</t>
+  </si>
+  <si>
+    <t>Explicação sobre ciclo de alta de juros e como ele favorece certas teses de renda fixa, ao mesmo tempo em que pressiona ativos de risco.</t>
+  </si>
+  <si>
+    <t>Discussão sobre ciclo de corte de juros e as oportunidades que surgem em duration, bolsa, crédito e reposicionamento gradual da carteira.</t>
+  </si>
+  <si>
+    <t>Contato de aniversário com tom próximo e consultivo, reforçando relacionamento e abrindo espaço para uma conversa de atualização patrimonial.</t>
+  </si>
+  <si>
+    <t>Retomada de contato com cliente que ficou mais distante, buscando reaquecer relacionamento e identificar mudanças recentes de contexto financeiro.</t>
+  </si>
+  <si>
+    <t>Mensagem de agradecimento pela indicação recebida, valorizando a confiança e fortalecendo o vínculo com o cliente indicador.</t>
+  </si>
+  <si>
+    <t>Convite para evento exclusivo com foco em estreitar relacionamento, gerar engajamento e abrir agenda para uma conversa mais estratégica.</t>
+  </si>
+  <si>
+    <t>Atualização trimestral para manter o cliente informado sobre carteira, cenário e próximos movimentos recomendados de forma recorrente.</t>
+  </si>
+  <si>
+    <t>Check-in semestral para revisar objetivos, carteira, percepções do cliente e possíveis ajustes no relacionamento ou na estratégia.</t>
+  </si>
+  <si>
+    <t>Follow-up após reunião para consolidar combinados, reforçar propostas discutidas e encaminhar próximos passos com clareza.</t>
+  </si>
+  <si>
+    <t>Estruturar um plano de aposentadoria com metas, prazo, aportes e alocação compatível com a renda futura desejada pelo cliente.</t>
+  </si>
+  <si>
+    <t>Conduzir conversa sobre sucessão patrimonial, eficiência na transmissão de patrimônio e instrumentos que apoiem essa organização.</t>
+  </si>
+  <si>
+    <t>Montar estratégia financeira para compra de imóvel, equilibrando segurança, liquidez e prazo do objetivo de aquisição.</t>
+  </si>
+  <si>
+    <t>Planejar a formação de recursos para educação dos filhos, distribuindo aportes e risco conforme a data esperada de uso do capital.</t>
+  </si>
+  <si>
+    <t>Desenhar uma rotina de aportes recorrentes que ajude o cliente a construir patrimônio com disciplina e consistência ao longo do tempo.</t>
+  </si>
+  <si>
+    <t>Estruturar um caminho para independência financeira, relacionando patrimônio-alvo, fluxo futuro desejado e ritmo de acumulação necessário.</t>
+  </si>
+  <si>
+    <t>Organizar investimentos para viabilizar viagem relevante ou projeto pessoal, respeitando orçamento, prazo e liquidez da meta.</t>
+  </si>
+  <si>
+    <t>Planejar uma carteira voltada à geração de renda passiva, com foco em previsibilidade de fluxo e equilíbrio entre risco e retorno.</t>
+  </si>
+  <si>
+    <t>Preparar financeiramente uma mudança de país, considerando moeda, liquidez, custos de transição e exposição internacional.</t>
+  </si>
+  <si>
+    <t>Planejar a alocação e o uso estratégico de recursos ligados à futura venda de empresa, com atenção a liquidez e preservação patrimonial.</t>
+  </si>
+  <si>
+    <t>Sugerir mecanismos de proteção cambial para reduzir impacto de oscilações do dólar sobre patrimônio, passivos ou objetivos em moeda forte.</t>
+  </si>
+  <si>
+    <t>Ajustar a carteira para reduzir oscilações, priorizando combinação de ativos mais estáveis e menor sensibilidade a choques de mercado.</t>
+  </si>
+  <si>
+    <t>Introduzir proteções contra inflação, buscando preservar poder de compra do patrimônio em cenários de pressão de preços.</t>
+  </si>
+  <si>
+    <t>Montar defesa da carteira para cenários de crise, combinando diversificação, liquidez e ativos menos correlacionados ao risco local.</t>
+  </si>
+  <si>
+    <t>Redesenhar a carteira para espalhar melhor os riscos entre classes, geografias, emissores e estratégias de investimento.</t>
+  </si>
+  <si>
+    <t>Reduzir exposição a emissores ou estruturas de crédito mais sensíveis, aumentando a robustez da carteira em renda fixa.</t>
+  </si>
+  <si>
+    <t>Revisar carteira com desempenho abaixo da referência para identificar causas, corrigir desvios e redefinir próximos passos de alocação.</t>
+  </si>
+  <si>
+    <t>Discutir realização parcial ou total de lucros após valorização relevante, transformando ganho potencial em ganho efetivamente capturado.</t>
+  </si>
+  <si>
+    <t>Revisão mais ampla da estratégia de investimento para verificar se a execução ainda faz sentido diante dos objetivos e do cenário atual.</t>
+  </si>
+  <si>
+    <t>Aproveitar um momento de alta de mercado para avaliar rebalanceamento, realização seletiva ou reforço de posições vencedoras.</t>
+  </si>
+  <si>
+    <t>Reposicionar a carteira após perdas relevantes, buscando recuperar coerência estratégica sem decisões precipitadas ou emocionais.</t>
+  </si>
+  <si>
+    <t>Explicação didática sobre tributação de investimentos, cobrindo incidência de imposto, prazos e impacto no retorno líquido do cliente.</t>
+  </si>
+  <si>
+    <t>Explicação detalhada sobre produto estruturado, mostrando montagem, cenários possíveis, riscos, prazos e forma de remuneração.</t>
+  </si>
+  <si>
+    <t>Conteúdo educativo sobre como funciona um fundo de investimento, incluindo cotas, gestão, taxas, risco e papel na carteira.</t>
+  </si>
+  <si>
+    <t>Explicação comparativa entre renda fixa e renda variável, ajudando o cliente a entender risco, previsibilidade e potencial de retorno.</t>
+  </si>
+  <si>
+    <t>Orientação sobre diversificação de carteira, mostrando por que combinar classes e estratégias reduz dependência de uma única tese.</t>
+  </si>
+  <si>
+    <t>Explicação sobre estratégias de longo prazo e como constância, horizonte e disciplina influenciam o resultado do investimento.</t>
+  </si>
+  <si>
+    <t>Solicitação para atualizar o perfil de suitability e garantir que futuras recomendações continuem aderentes às exigências regulatórias.</t>
+  </si>
+  <si>
+    <t>Contato para revisar dados cadastrais do cliente, assegurando consistência documental e continuidade operacional da conta.</t>
+  </si>
+  <si>
+    <t>Validação do perfil de risco do cliente antes de novas recomendações, confirmando aderência entre tolerância a risco e estratégia proposta.</t>
   </si>
 </sst>
 </file>
@@ -1127,6 +1283,7 @@
   <dimension ref="A1:E79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="39.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1161,12 +1318,12 @@
         <v>7</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>70</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>8</v>
@@ -1178,12 +1335,12 @@
         <v>9</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>72</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>10</v>
@@ -1195,12 +1352,12 @@
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>74</v>
+        <v>231</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>
@@ -1212,12 +1369,12 @@
         <v>13</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>76</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>14</v>
@@ -1229,66 +1386,66 @@
         <v>15</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>78</v>
+        <v>233</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>82</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>86</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>90</v>
+        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>6</v>
@@ -1297,165 +1454,165 @@
         <v>58</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>93</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>97</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>101</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>103</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>21</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>105</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>109</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>113</v>
+        <v>243</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>117</v>
+        <v>244</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>121</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>125</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>126</v>
+        <v>108</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>22</v>
@@ -1467,12 +1624,12 @@
         <v>23</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>127</v>
+        <v>247</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>24</v>
@@ -1484,12 +1641,12 @@
         <v>25</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>127</v>
+        <v>248</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>26</v>
@@ -1501,12 +1658,12 @@
         <v>27</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>127</v>
+        <v>249</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>28</v>
@@ -1518,12 +1675,12 @@
         <v>29</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>127</v>
+        <v>250</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>30</v>
@@ -1535,12 +1692,12 @@
         <v>31</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>127</v>
+        <v>251</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>32</v>
@@ -1552,12 +1709,12 @@
         <v>33</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>127</v>
+        <v>252</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>34</v>
@@ -1569,83 +1726,83 @@
         <v>35</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>127</v>
+        <v>253</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>135</v>
+        <v>116</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>136</v>
+        <v>117</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>127</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>127</v>
+        <v>255</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>127</v>
+        <v>256</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>145</v>
+        <v>126</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>127</v>
+        <v>257</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>66</v>
@@ -1654,199 +1811,199 @@
         <v>25</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>127</v>
+        <v>258</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>127</v>
+        <v>259</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>153</v>
+        <v>134</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>127</v>
+        <v>260</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>154</v>
+        <v>135</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>66</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>127</v>
+        <v>261</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>160</v>
+        <v>262</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>162</v>
+        <v>142</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>160</v>
+        <v>263</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>163</v>
+        <v>143</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>39</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>160</v>
+        <v>264</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>164</v>
+        <v>144</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>166</v>
+        <v>146</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>160</v>
+        <v>265</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>168</v>
+        <v>148</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>160</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>169</v>
+        <v>149</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>171</v>
+        <v>151</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>160</v>
+        <v>267</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>160</v>
+        <v>268</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>176</v>
+        <v>156</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>160</v>
+        <v>269</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>40</v>
@@ -1858,12 +2015,12 @@
         <v>41</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>179</v>
+        <v>270</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>180</v>
+        <v>159</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>42</v>
@@ -1875,12 +2032,12 @@
         <v>43</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>179</v>
+        <v>271</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>181</v>
+        <v>160</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>44</v>
@@ -1892,12 +2049,12 @@
         <v>45</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>179</v>
+        <v>272</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>182</v>
+        <v>161</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>46</v>
@@ -1909,32 +2066,32 @@
         <v>47</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>179</v>
+        <v>273</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>183</v>
+        <v>162</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>41</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>179</v>
+        <v>274</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>41</v>
@@ -1943,15 +2100,15 @@
         <v>41</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>179</v>
+        <v>275</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
-        <v>187</v>
+        <v>166</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>41</v>
@@ -1960,12 +2117,12 @@
         <v>41</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>179</v>
+        <v>276</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>189</v>
+        <v>168</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>48</v>
@@ -1977,12 +2134,12 @@
         <v>50</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>190</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>191</v>
+        <v>169</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>51</v>
@@ -1994,12 +2151,12 @@
         <v>52</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>190</v>
+        <v>278</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>53</v>
@@ -2008,52 +2165,52 @@
         <v>49</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>190</v>
+        <v>279</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>194</v>
+        <v>172</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>195</v>
+        <v>173</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>190</v>
+        <v>280</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>190</v>
+        <v>281</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>49</v>
@@ -2062,32 +2219,32 @@
         <v>50</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>190</v>
+        <v>282</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>190</v>
+        <v>283</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>49</v>
@@ -2096,15 +2253,15 @@
         <v>17</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>190</v>
+        <v>284</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>49</v>
@@ -2113,29 +2270,29 @@
         <v>31</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>190</v>
+        <v>285</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>190</v>
+        <v>286</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>54</v>
@@ -2147,12 +2304,12 @@
         <v>56</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>212</v>
+        <v>287</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
-        <v>213</v>
+        <v>190</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>57</v>
@@ -2164,15 +2321,15 @@
         <v>58</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>212</v>
+        <v>288</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
-        <v>214</v>
+        <v>191</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>215</v>
+        <v>192</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>55</v>
@@ -2181,15 +2338,15 @@
         <v>56</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>212</v>
+        <v>289</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
-        <v>216</v>
+        <v>193</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>217</v>
+        <v>194</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>55</v>
@@ -2198,15 +2355,15 @@
         <v>58</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>212</v>
+        <v>290</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
-        <v>218</v>
+        <v>195</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>219</v>
+        <v>196</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>55</v>
@@ -2215,46 +2372,46 @@
         <v>11</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>212</v>
+        <v>291</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
-        <v>220</v>
+        <v>197</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>221</v>
+        <v>198</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>55</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>212</v>
+        <v>292</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>223</v>
+        <v>200</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>59</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>225</v>
+        <v>293</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
-        <v>226</v>
+        <v>202</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>60</v>
@@ -2266,32 +2423,32 @@
         <v>61</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>225</v>
+        <v>294</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>227</v>
+        <v>203</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>59</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>229</v>
+        <v>205</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>225</v>
+        <v>295</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
-        <v>230</v>
+        <v>206</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>231</v>
+        <v>207</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>59</v>
@@ -2300,29 +2457,29 @@
         <v>62</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>225</v>
+        <v>296</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>232</v>
+        <v>208</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>233</v>
+        <v>209</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>59</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>234</v>
+        <v>210</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>225</v>
+        <v>297</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>63</v>
@@ -2331,15 +2488,15 @@
         <v>64</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>236</v>
+        <v>212</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>237</v>
+        <v>298</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
-        <v>238</v>
+        <v>213</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>65</v>
@@ -2351,80 +2508,80 @@
         <v>66</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>237</v>
+        <v>299</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
-        <v>239</v>
+        <v>214</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>237</v>
+        <v>300</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
-        <v>242</v>
+        <v>217</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>243</v>
+        <v>218</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>237</v>
+        <v>301</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
-        <v>244</v>
+        <v>219</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>245</v>
+        <v>220</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>237</v>
+        <v>302</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
-        <v>246</v>
+        <v>221</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>247</v>
+        <v>222</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>241</v>
+        <v>216</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>237</v>
+        <v>303</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
-        <v>248</v>
+        <v>223</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>67</v>
@@ -2433,18 +2590,18 @@
         <v>68</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>249</v>
+        <v>224</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>250</v>
+        <v>304</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
-        <v>251</v>
+        <v>225</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>252</v>
+        <v>226</v>
       </c>
       <c r="C78" s="1" t="s">
         <v>68</v>
@@ -2453,15 +2610,15 @@
         <v>68</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>250</v>
+        <v>305</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
-        <v>253</v>
+        <v>227</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>254</v>
+        <v>228</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>68</v>
@@ -2470,7 +2627,7 @@
         <v>68</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>250</v>
+        <v>306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>